<commit_message>
Use Etagi txt templates for device xlsx without splitting text
- Add template_engine: load txt, fill {{placeholders}}, write line-by-line to xlsx
- Support card, checklist, and daily report templates
- Default templates in input/templates/ until user uploads their files
- Also save rendered .txt copy for each device document

Co-authored-by: sniper072 <sniper072@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/equipment-templates/output/checklists/TEST_Checklist_67plus_LS67Y43279.xlsx
+++ b/equipment-templates/output/checklists/TEST_Checklist_67plus_LS67Y43279.xlsx
@@ -17,13 +17,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +50,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,350 +420,208 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:A31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>№</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Пункт проверки</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Да / Нет</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Фактическое значение</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Примечание</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ЧЕК-ЛИСТ ПРОВЕРКИ ОРГТЕХНИКИ</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Инвентарный номер</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>67+</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Организация: Этажи</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Модель</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Kyocera ECOSYS M3040dn</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="A3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Серийный номер</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>LS67Y43279</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Дата проверки: 22.06.2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Местоположение</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Риелторы (Тюмень)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="A5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Дата проверки</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>22.06.2026</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Инвентарный номер: 67+</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Модель соответствует учетным данным</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Kyocera ECOSYS M3040dn</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Модель: Kyocera ECOSYS M3040dn</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Серийный номер соответствует</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>LS67Y43279</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Серийный номер: LS67Y43279</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Инвентарный номер соответствует</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>67+</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Местоположение: Риелторы (Тюмень)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Место размещения соответствует</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Риелторы (Тюмень)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Офис: Тюмень</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Офис соответствует</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Тюмень</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Подразделение: Риелторы</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Подразделение соответствует</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Риелторы</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+      <c r="A12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Показания счетчика за предыдущий месяц зафиксированы</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>272339</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Проверка:</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Показания счетчика за отчетный месяц зафиксированы</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>272864</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Модель соответствует учетным данным. Факт: Kyocera ECOSYS M3040dn</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Количество отпечатков за период проверено</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>525</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Серийный номер соответствует. Факт: LS67Y43279</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Устройство включено и исправно</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Инвентарный номер соответствует. Факт: 67+</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Печать / сканирование выполняется</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Место размещения соответствует. Факт: Риелторы (Тюмень)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Ответственный сотрудник определен</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Офис соответствует. Факт: Тюмень</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Внешний вид и комплектность в норме</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Подразделение соответствует. Факт: Риелторы</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Замечания отсутствуют</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Счетчик (предыдущий месяц) зафиксирован. Факт: 272339</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Проверил</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Счетчик (отчетный месяц) зафиксирован. Факт: 272864</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Подпись ответственного</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Кол-во отпечатков проверено. Факт: 525</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Устройство включено и исправно</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Печать / сканирование выполняется</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[ ] Ответственный сотрудник определен. Факт: </t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Внешний вид и комплектность в норме</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
+          <t>[ ] Замечания отсутствуют</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
+        <is>
+          <t>Проверил: __________________ / __________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Подпись ответственного: __________________</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>